<commit_message>
Refresh publications data from OpenAlex
Automated weekly refresh.
</commit_message>
<xml_diff>
--- a/papers.xlsx
+++ b/papers.xlsx
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>

</xml_diff>